<commit_message>
cambios final del día
</commit_message>
<xml_diff>
--- a/intermedios/2. tamanio_de_muestra/resultado00.xlsx
+++ b/intermedios/2. tamanio_de_muestra/resultado00.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ppenafiel\Desktop\PRODUCTOS NUEVOS\NUEVA_ENEMDU_2024\Tratadas\2. tamaño_de_muestra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nueva_ENEMDU\intermedios\2. tamanio_de_muestra\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="resultados_desemp" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="84">
   <si>
     <t>dominio</t>
   </si>
@@ -243,33 +243,6 @@
     <t>2513</t>
   </si>
   <si>
-    <t>1211</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>1212</t>
-  </si>
-  <si>
-    <t>1213</t>
-  </si>
-  <si>
-    <t>1221</t>
-  </si>
-  <si>
-    <t>1222</t>
-  </si>
-  <si>
-    <t>1223</t>
-  </si>
-  <si>
-    <t>Mi</t>
-  </si>
-  <si>
-    <t>Mih</t>
-  </si>
-  <si>
     <t>eabs= error estandar</t>
   </si>
   <si>
@@ -433,8 +406,8 @@
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="115224" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1"/>
@@ -470,6 +443,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -502,7 +476,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1"/>
@@ -927,22 +901,22 @@
         <v>53</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
@@ -7492,10 +7466,10 @@
         <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -8208,10 +8182,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
@@ -8219,13 +8196,13 @@
         <v>62</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
@@ -8234,20 +8211,12 @@
       <c r="J1" s="23"/>
       <c r="K1" s="23"/>
       <c r="L1" s="23"/>
-      <c r="P1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -8289,28 +8258,9 @@
         <f>MAX(G2,L2)</f>
         <v>4</v>
       </c>
-      <c r="P2" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>74</v>
-      </c>
-      <c r="R2">
-        <v>51545</v>
-      </c>
-      <c r="S2">
-        <f>15*(R2/$R$8)</f>
-        <v>4.075906459877487</v>
-      </c>
-      <c r="T2" s="2">
-        <f>ROUNDUP(MAX(S2),0)</f>
-        <v>5</v>
-      </c>
-      <c r="U2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T2" s="2"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -8352,28 +8302,9 @@
         <f t="shared" ref="M3:M10" si="3">MAX(G3,L3)</f>
         <v>4</v>
       </c>
-      <c r="P3" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>74</v>
-      </c>
-      <c r="R3">
-        <v>32417</v>
-      </c>
-      <c r="S3">
-        <f t="shared" ref="S3:S7" si="4">15*(R3/$R$8)</f>
-        <v>2.5633652092317103</v>
-      </c>
-      <c r="T3" s="2">
-        <f t="shared" ref="T3:T7" si="5">ROUNDUP(MAX(S3),0)</f>
-        <v>3</v>
-      </c>
-      <c r="U3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T3" s="2"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>66</v>
       </c>
@@ -8415,28 +8346,9 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="P4" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>74</v>
-      </c>
-      <c r="R4">
-        <v>36931</v>
-      </c>
-      <c r="S4">
-        <f t="shared" si="4"/>
-        <v>2.9203084968422828</v>
-      </c>
-      <c r="T4" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="U4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T4" s="2"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -8478,28 +8390,9 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="P5" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>74</v>
-      </c>
-      <c r="R5">
-        <v>33232</v>
-      </c>
-      <c r="S5">
-        <f t="shared" si="4"/>
-        <v>2.6278111063080538</v>
-      </c>
-      <c r="T5" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="U5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T5" s="2"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -8541,28 +8434,9 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="P6" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>74</v>
-      </c>
-      <c r="R6">
-        <v>29457</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="4"/>
-        <v>2.3293040370280558</v>
-      </c>
-      <c r="T6" s="2">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="U6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T6" s="2"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -8604,28 +8478,9 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="P7" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>74</v>
-      </c>
-      <c r="R7">
-        <v>6112</v>
-      </c>
-      <c r="S7">
-        <f t="shared" si="4"/>
-        <v>0.48330469071241056</v>
-      </c>
-      <c r="T7" s="2">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="U7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="T7" s="2"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>70</v>
       </c>
@@ -8664,18 +8519,14 @@
         <v>12.221342864437069</v>
       </c>
       <c r="L8" s="24">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M8">
         <f t="shared" si="3"/>
-        <v>12</v>
-      </c>
-      <c r="R8">
-        <f>SUM(R2:R7)</f>
-        <v>189694</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>71</v>
       </c>
@@ -8703,14 +8554,14 @@
         <v>202152</v>
       </c>
       <c r="I9" s="24">
-        <f t="shared" ref="I9:I10" si="6">H9/$H$11</f>
+        <f t="shared" ref="I9:I10" si="4">H9/$H$11</f>
         <v>0.42651970537411621</v>
       </c>
       <c r="J9" s="24">
         <v>33</v>
       </c>
       <c r="K9" s="24">
-        <f t="shared" ref="K9:K10" si="7">I9*J9</f>
+        <f t="shared" ref="K9:K10" si="5">I9*J9</f>
         <v>14.075150277345834</v>
       </c>
       <c r="L9" s="24">
@@ -8721,7 +8572,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>72</v>
       </c>
@@ -8749,14 +8600,14 @@
         <v>96278</v>
       </c>
       <c r="I10" s="24">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>0.2031365714611241</v>
       </c>
       <c r="J10" s="24">
         <v>33</v>
       </c>
       <c r="K10" s="24">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>6.7035068582170956</v>
       </c>
       <c r="L10" s="24">
@@ -8767,13 +8618,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C11">
         <f>SUM(C2:C10)</f>
         <v>732845</v>
       </c>
       <c r="H11">
         <f>SUM(H8:H10)</f>
+        <v>473957</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D12" s="20">
+        <f>C8/C13</f>
+        <v>0.37034372316475966</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <f>SUM(C8:C10)</f>
         <v>473957</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PP JN RE: calculo de muestra desempleo desocupacion desde el censo
</commit_message>
<xml_diff>
--- a/intermedios/2. tamanio_de_muestra/resultado00.xlsx
+++ b/intermedios/2. tamanio_de_muestra/resultado00.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="3"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="resultados_desemp" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="85">
   <si>
     <t>dominio</t>
   </si>
@@ -275,6 +275,9 @@
   <si>
     <t>muestra_pichincha</t>
   </si>
+  <si>
+    <t>afinamiento</t>
+  </si>
 </sst>
 </file>
 
@@ -309,7 +312,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -334,6 +337,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -348,7 +363,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -378,6 +393,20 @@
     <xf numFmtId="166" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4665,15 +4694,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="20.28515625" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="10" width="9.140625" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="28" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="26" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" customWidth="1"/>
     <col min="15" max="17" width="13.28515625" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="20" max="21" width="9.140625" customWidth="1"/>
+    <col min="22" max="22" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4704,13 +4742,13 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="29" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="25" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -4737,8 +4775,11 @@
       <c r="U1" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V1" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -4769,18 +4810,18 @@
       <c r="J2">
         <v>104713</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="34">
         <v>6.7753477838887104</v>
       </c>
       <c r="L2">
         <v>345174</v>
       </c>
-      <c r="M2">
-        <v>3.2963815381089261</v>
+      <c r="M2" s="32">
+        <v>3.2963815381089301</v>
       </c>
       <c r="N2">
         <f>(H2-1)/(K2*M2-1)</f>
-        <v>0.80214186928869724</v>
+        <v>0.80214186928869613</v>
       </c>
       <c r="O2">
         <f>C2*(1-C2)*H2</f>
@@ -4811,7 +4852,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -4842,13 +4883,13 @@
       <c r="J3">
         <v>77573</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="34">
         <v>6.7903536414565826</v>
       </c>
       <c r="L3">
         <v>252463</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="32">
         <v>3.2545215474456319</v>
       </c>
       <c r="N3">
@@ -4884,7 +4925,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -4915,13 +4956,13 @@
       <c r="J4">
         <v>27140</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="34">
         <v>6.7328206400396926</v>
       </c>
       <c r="L4">
         <v>92711</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="32">
         <v>3.4160280029476788</v>
       </c>
       <c r="N4">
@@ -4957,7 +4998,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -4988,13 +5029,13 @@
       <c r="J5">
         <v>9508</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="34">
         <v>6.8304597701149428</v>
       </c>
       <c r="L5">
         <v>30407</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="32">
         <v>3.1980437526293648</v>
       </c>
       <c r="N5">
@@ -5030,7 +5071,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -5061,13 +5102,13 @@
       <c r="J6">
         <v>1906</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="34">
         <v>6.6180555555555554</v>
       </c>
       <c r="L6">
         <v>5827</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="32">
         <v>3.0571878279118572</v>
       </c>
       <c r="N6">
@@ -5103,7 +5144,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -5134,13 +5175,13 @@
       <c r="J7">
         <v>1946</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="34">
         <v>6.7569444444444446</v>
       </c>
       <c r="L7">
         <v>6212</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="32">
         <v>3.1921891058581711</v>
       </c>
       <c r="N7">
@@ -5176,7 +5217,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -5207,13 +5248,13 @@
       <c r="J8">
         <v>2302</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="34">
         <v>6.8511904761904763</v>
       </c>
       <c r="L8">
         <v>7411</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="32">
         <v>3.219374456993918</v>
       </c>
       <c r="N8">
@@ -5249,7 +5290,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -5280,13 +5321,13 @@
       <c r="J9">
         <v>1936</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="34">
         <v>6.7222222222222223</v>
       </c>
       <c r="L9">
         <v>6124</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="32">
         <v>3.1632231404958682</v>
       </c>
       <c r="N9">
@@ -5322,80 +5363,80 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="27">
         <v>5712</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="27">
         <v>0.31019999999999998</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="27">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="27">
         <v>1.893</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="27">
         <v>27.309000000000001</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="27">
         <v>34.729999999999997</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="27">
         <v>9.577</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="27">
         <v>470596</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="27">
         <v>1930</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="30">
         <v>6.7013888888888893</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="27">
         <v>5712</v>
       </c>
-      <c r="M10">
-        <v>2.959585492227979</v>
-      </c>
-      <c r="N10">
-        <f t="shared" si="1"/>
-        <v>0.45541592920353985</v>
-      </c>
-      <c r="O10">
+      <c r="M10" s="30">
+        <v>2.9595854922279798</v>
+      </c>
+      <c r="N10" s="27">
+        <f t="shared" si="1"/>
+        <v>0.45541592920353968</v>
+      </c>
+      <c r="O10" s="27">
         <f t="shared" si="2"/>
         <v>2.0492477689199995</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="27">
         <f t="shared" si="3"/>
         <v>2.4032918649769495E-3</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="27">
         <f t="shared" si="4"/>
         <v>1.25</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="30">
         <f t="shared" si="0"/>
         <v>852.68368723066192</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="31">
         <f t="shared" si="5"/>
         <v>853</v>
       </c>
-      <c r="T10">
+      <c r="T10" s="27">
         <f t="shared" si="6"/>
         <v>289</v>
       </c>
-      <c r="U10">
+      <c r="U10" s="27">
         <f t="shared" si="7"/>
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -5426,13 +5467,13 @@
       <c r="J11">
         <v>11179</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="34">
         <v>6.8498774509803919</v>
       </c>
       <c r="L11">
         <v>36493</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="32">
         <v>3.264424367116916</v>
       </c>
       <c r="N11">
@@ -5468,80 +5509,80 @@
         <v>176</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:22" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="26">
         <v>21802</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="26">
         <v>0.45638000000000001</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="26">
         <v>0.02</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="26">
         <v>0.90600000000000003</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="26">
         <v>43.860999999999997</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="26">
         <v>47.414000000000001</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="26">
         <v>7.399</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="26">
         <v>550425</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="26">
         <v>6135</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="32">
         <v>6.7269736842105274</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="26">
         <v>21802</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="32">
         <v>3.5537082314588431</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="26">
         <f t="shared" si="1"/>
         <v>0.27936275730014354</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="26">
         <f t="shared" si="2"/>
         <v>1.8356718901444</v>
       </c>
-      <c r="P12">
+      <c r="P12" s="26">
         <f t="shared" si="3"/>
         <v>5.1959786082030153E-3</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="26">
         <f t="shared" si="4"/>
         <v>1.25</v>
       </c>
-      <c r="R12" s="3">
+      <c r="R12" s="32">
         <f t="shared" si="0"/>
         <v>353.28703764222223</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="33">
         <f t="shared" si="5"/>
         <v>354</v>
       </c>
-      <c r="T12">
+      <c r="T12" s="26">
         <f t="shared" si="6"/>
         <v>100</v>
       </c>
-      <c r="U12">
+      <c r="U12" s="26">
         <f t="shared" si="7"/>
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -5572,13 +5613,13 @@
       <c r="J13">
         <v>12660</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="34">
         <v>6.7628205128205128</v>
       </c>
       <c r="L13">
         <v>44034</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="32">
         <v>3.4781990521327009</v>
       </c>
       <c r="N13">
@@ -5614,7 +5655,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -5645,13 +5686,13 @@
       <c r="J14">
         <v>4926</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="34">
         <v>6.8416666666666668</v>
       </c>
       <c r="L14">
         <v>16337</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="32">
         <v>3.3164839626471778</v>
       </c>
       <c r="N14">
@@ -5687,7 +5728,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -5718,13 +5759,13 @@
       <c r="J15">
         <v>3559</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="34">
         <v>6.7405303030303028</v>
       </c>
       <c r="L15">
         <v>11376</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="32">
         <v>3.1964034841247542</v>
       </c>
       <c r="N15">
@@ -5760,7 +5801,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -5791,13 +5832,13 @@
       <c r="J16">
         <v>1933</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="34">
         <v>6.7118055555555554</v>
       </c>
       <c r="L16">
         <v>6431</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="32">
         <v>3.3269529229177439</v>
       </c>
       <c r="N16">
@@ -5864,13 +5905,13 @@
       <c r="J17">
         <v>2268</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="34">
         <v>6.75</v>
       </c>
       <c r="L17">
         <v>7642</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="32">
         <v>3.3694885361552029</v>
       </c>
       <c r="N17">
@@ -5937,13 +5978,13 @@
       <c r="J18">
         <v>1285</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="34">
         <v>6.692708333333333</v>
       </c>
       <c r="L18">
         <v>4676</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="32">
         <v>3.6389105058365758</v>
       </c>
       <c r="N18">
@@ -6010,13 +6051,13 @@
       <c r="J19">
         <v>1585</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="34">
         <v>6.6317991631799167</v>
       </c>
       <c r="L19">
         <v>5888</v>
       </c>
-      <c r="M19">
+      <c r="M19" s="32">
         <v>3.7148264984227128</v>
       </c>
       <c r="N19">
@@ -6083,13 +6124,13 @@
       <c r="J20">
         <v>1928</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="34">
         <v>6.6944444444444446</v>
       </c>
       <c r="L20">
         <v>6855</v>
       </c>
-      <c r="M20">
+      <c r="M20" s="32">
         <v>3.5554979253112031</v>
       </c>
       <c r="N20">
@@ -6125,75 +6166,75 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:21" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="27">
         <v>47254</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="27">
         <v>0.11301</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="27">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="27">
         <v>0.39900000000000002</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="27">
         <v>10.52</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="27">
         <v>12.083</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="27">
         <v>7.51</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="27">
         <v>3083707</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="27">
         <v>15369</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="30">
         <v>6.8125</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="27">
         <v>47254</v>
       </c>
-      <c r="M21">
+      <c r="M21" s="30">
         <v>3.074630750211464</v>
       </c>
-      <c r="N21">
+      <c r="N21" s="27">
         <f t="shared" si="1"/>
         <v>0.32638250588915069</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="27">
         <f t="shared" si="2"/>
         <v>0.75279293664899993</v>
       </c>
-      <c r="P21">
+      <c r="P21" s="27">
         <f t="shared" si="3"/>
         <v>3.1864118568087957E-4</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="27">
         <f t="shared" si="4"/>
         <v>1.25</v>
       </c>
-      <c r="R21" s="3">
+      <c r="R21" s="30">
         <f t="shared" si="0"/>
         <v>2362.5098401526948</v>
       </c>
-      <c r="S21" s="2">
+      <c r="S21" s="31">
         <f t="shared" si="5"/>
         <v>2363</v>
       </c>
-      <c r="T21">
+      <c r="T21" s="27">
         <f t="shared" si="6"/>
         <v>769</v>
       </c>
-      <c r="U21">
+      <c r="U21" s="27">
         <f t="shared" si="7"/>
         <v>110</v>
       </c>
@@ -6229,13 +6270,13 @@
       <c r="J22">
         <v>8854</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="34">
         <v>6.8317901234567904</v>
       </c>
       <c r="L22">
         <v>26259</v>
       </c>
-      <c r="M22">
+      <c r="M22" s="32">
         <v>2.9657781793539639</v>
       </c>
       <c r="N22">
@@ -6302,13 +6343,13 @@
       <c r="J23">
         <v>1951</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="34">
         <v>6.7743055555555554</v>
       </c>
       <c r="L23">
         <v>6677</v>
       </c>
-      <c r="M23">
+      <c r="M23" s="32">
         <v>3.4223475140953359</v>
       </c>
       <c r="N23">
@@ -6375,13 +6416,13 @@
       <c r="J24">
         <v>1223</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="34">
         <v>6.369791666666667</v>
       </c>
       <c r="L24">
         <v>3541</v>
       </c>
-      <c r="M24">
+      <c r="M24" s="32">
         <v>2.8953393295175802</v>
       </c>
       <c r="N24">
@@ -6448,13 +6489,13 @@
       <c r="J25">
         <v>2594</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="34">
         <v>6.755208333333333</v>
       </c>
       <c r="L25">
         <v>8925</v>
       </c>
-      <c r="M25">
+      <c r="M25" s="32">
         <v>3.4406322282189672</v>
       </c>
       <c r="N25">
@@ -6521,13 +6562,13 @@
       <c r="J26">
         <v>1923</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="34">
         <v>6.677083333333333</v>
       </c>
       <c r="L26">
         <v>7186</v>
       </c>
-      <c r="M26">
+      <c r="M26" s="32">
         <v>3.7368694747789908</v>
       </c>
       <c r="N26">
@@ -6563,75 +6604,75 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:21" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="27">
         <v>7165</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="27">
         <v>0.22856000000000001</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="27">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="27">
         <v>1.69</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="27">
         <v>19.542999999999999</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="27">
         <v>26.167999999999999</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="27">
         <v>11.702</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="27">
         <v>491394</v>
       </c>
-      <c r="J27">
+      <c r="J27" s="27">
         <v>2202</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="30">
         <v>6.5535714285714288</v>
       </c>
-      <c r="L27">
+      <c r="L27" s="27">
         <v>7165</v>
       </c>
-      <c r="M27">
+      <c r="M27" s="30">
         <v>3.2538601271571301</v>
       </c>
-      <c r="N27">
+      <c r="N27" s="27">
         <f t="shared" si="1"/>
         <v>0.52655908624981695</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="27">
         <f t="shared" si="2"/>
         <v>2.0633004595328002</v>
       </c>
-      <c r="P27">
+      <c r="P27" s="27">
         <f t="shared" si="3"/>
         <v>1.3065730059742694E-3</v>
       </c>
-      <c r="Q27">
+      <c r="Q27" s="27">
         <f t="shared" si="4"/>
         <v>1.25</v>
       </c>
-      <c r="R27" s="3">
+      <c r="R27" s="30">
         <f t="shared" si="0"/>
         <v>1579.1696675948572</v>
       </c>
-      <c r="S27" s="2">
+      <c r="S27" s="31">
         <f t="shared" si="5"/>
         <v>1580</v>
       </c>
-      <c r="T27">
+      <c r="T27" s="27">
         <f t="shared" si="6"/>
         <v>486</v>
       </c>
-      <c r="U27">
+      <c r="U27" s="27">
         <f t="shared" si="7"/>
         <v>70</v>
       </c>
@@ -6667,13 +6708,13 @@
       <c r="J28">
         <v>3611</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="34">
         <v>6.8390151515151514</v>
       </c>
       <c r="L28">
         <v>14940</v>
       </c>
-      <c r="M28">
+      <c r="M28" s="32">
         <v>4.1373580725560783</v>
       </c>
       <c r="N28">
@@ -6709,75 +6750,75 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:21" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="27">
         <v>26965</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="27">
         <v>7.7280000000000001E-2</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="27">
         <v>0.14000000000000001</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="27">
         <v>1.0840000000000001</v>
       </c>
-      <c r="F29" s="4">
+      <c r="F29" s="27">
         <v>5.6029999999999998</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29" s="27">
         <v>9.8529999999999998</v>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="27">
         <v>46.173000000000002</v>
       </c>
-      <c r="I29" s="4">
+      <c r="I29" s="27">
         <v>593830</v>
       </c>
-      <c r="J29" s="4">
+      <c r="J29" s="27">
         <v>8407</v>
       </c>
-      <c r="K29" s="4">
+      <c r="K29" s="30">
         <v>6.8516707416462914</v>
       </c>
-      <c r="L29" s="4">
+      <c r="L29" s="27">
         <v>26965</v>
       </c>
-      <c r="M29" s="4">
+      <c r="M29" s="30">
         <v>3.2074461758058761</v>
       </c>
-      <c r="N29" s="4">
+      <c r="N29" s="27">
         <f t="shared" si="1"/>
         <v>2.1535189602921752</v>
       </c>
-      <c r="O29" s="4">
+      <c r="O29" s="27">
         <f t="shared" si="2"/>
         <v>3.2924951232768001</v>
       </c>
-      <c r="P29" s="4">
+      <c r="P29" s="27">
         <f t="shared" si="3"/>
         <v>1.5443588074816699E-4</v>
       </c>
-      <c r="Q29" s="4">
+      <c r="Q29" s="27">
         <f t="shared" si="4"/>
         <v>1.25</v>
       </c>
-      <c r="R29" s="5">
+      <c r="R29" s="30">
         <f t="shared" si="0"/>
         <v>21319.495879624974</v>
       </c>
-      <c r="S29" s="6">
+      <c r="S29" s="31">
         <f t="shared" si="5"/>
         <v>21320</v>
       </c>
-      <c r="T29" s="4">
+      <c r="T29" s="27">
         <f t="shared" si="6"/>
         <v>6648</v>
       </c>
-      <c r="U29" s="4">
+      <c r="U29" s="27">
         <f t="shared" si="7"/>
         <v>950</v>
       </c>
@@ -6813,13 +6854,13 @@
       <c r="J30">
         <v>941</v>
       </c>
-      <c r="K30">
+      <c r="K30" s="34">
         <v>6.7697841726618702</v>
       </c>
       <c r="L30">
         <v>2800</v>
       </c>
-      <c r="M30">
+      <c r="M30" s="32">
         <v>2.9755579171094579</v>
       </c>
       <c r="N30">
@@ -6886,13 +6927,13 @@
       <c r="J31">
         <v>1599</v>
       </c>
-      <c r="K31">
+      <c r="K31" s="34">
         <v>6.7184873949579833</v>
       </c>
       <c r="L31">
         <v>5234</v>
       </c>
-      <c r="M31">
+      <c r="M31" s="32">
         <v>3.273295809881176</v>
       </c>
       <c r="N31">
@@ -6959,13 +7000,13 @@
       <c r="J32">
         <v>14009</v>
       </c>
-      <c r="K32">
+      <c r="K32" s="34">
         <v>6.8070942662779386</v>
       </c>
       <c r="L32">
         <v>42768</v>
       </c>
-      <c r="M32">
+      <c r="M32" s="32">
         <v>3.0528945677778569</v>
       </c>
       <c r="N32">
@@ -7032,13 +7073,13 @@
       <c r="J33">
         <v>7634</v>
       </c>
-      <c r="K33">
+      <c r="K33" s="34">
         <v>6.834377797672337</v>
       </c>
       <c r="L33">
         <v>22503</v>
       </c>
-      <c r="M33">
+      <c r="M33" s="32">
         <v>2.9477338223735918</v>
       </c>
       <c r="N33">
@@ -7105,13 +7146,13 @@
       <c r="J34">
         <v>1969</v>
       </c>
-      <c r="K34">
+      <c r="K34" s="34">
         <v>6.5633333333333326</v>
       </c>
       <c r="L34">
         <v>6451</v>
       </c>
-      <c r="M34">
+      <c r="M34" s="32">
         <v>3.2762823768410358</v>
       </c>
       <c r="N34">
@@ -7178,13 +7219,13 @@
       <c r="J35">
         <v>8568</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="34">
         <v>6.865384615384615</v>
       </c>
       <c r="L35">
         <v>28158</v>
       </c>
-      <c r="M35">
+      <c r="M35" s="32">
         <v>3.28641456582633</v>
       </c>
       <c r="N35">
@@ -7251,13 +7292,13 @@
       <c r="J36">
         <v>2002</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="34">
         <v>6.7635135135135132</v>
       </c>
       <c r="L36">
         <v>6968</v>
       </c>
-      <c r="M36">
+      <c r="M36" s="32">
         <v>3.4805194805194799</v>
       </c>
       <c r="N36">
@@ -7324,13 +7365,13 @@
       <c r="J37">
         <v>10450</v>
       </c>
-      <c r="K37">
+      <c r="K37" s="34">
         <v>6.7593790426908154</v>
       </c>
       <c r="L37">
         <v>36509</v>
       </c>
-      <c r="M37">
+      <c r="M37" s="32">
         <v>3.4936842105263159</v>
       </c>
       <c r="N37">
@@ -7397,13 +7438,13 @@
       <c r="J38">
         <v>343</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="34">
         <v>6.86</v>
       </c>
       <c r="L38">
         <v>1268</v>
       </c>
-      <c r="M38">
+      <c r="M38" s="32">
         <v>3.6967930029154519</v>
       </c>
       <c r="N38">

</xml_diff>